<commit_message>
Updated anon data for location
</commit_message>
<xml_diff>
--- a/anonymized_data/crm_anonymized_data.xlsx
+++ b/anonymized_data/crm_anonymized_data.xlsx
@@ -2886,12 +2886,12 @@
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>Paulbury</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="I2" s="7" t="inlineStr">
         <is>
-          <t>college</t>
+          <t>other</t>
         </is>
       </c>
       <c r="J2" s="11" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="H3" s="8" t="inlineStr">
         <is>
-          <t>Christinaland</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="I3" s="8" t="inlineStr">
@@ -2980,12 +2980,12 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>Tylerborough</t>
+          <t>Washington D.C.</t>
         </is>
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>other</t>
         </is>
       </c>
       <c r="J4" s="11" t="n">
@@ -3027,12 +3027,12 @@
       </c>
       <c r="H5" s="12" t="inlineStr">
         <is>
-          <t>New Travis</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>college</t>
         </is>
       </c>
       <c r="J5" s="19" t="n">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Joseshire</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="I6" s="8" t="inlineStr">
@@ -3121,12 +3121,12 @@
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
-          <t>Millerland</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="I7" s="8" t="inlineStr">
         <is>
-          <t>cold outreach</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="J7" s="19" t="n">
@@ -3168,12 +3168,12 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>West Oliviashire</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>cold outreach</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="J8" s="11" t="n">
@@ -3215,12 +3215,12 @@
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t>Williamton</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>life</t>
         </is>
       </c>
       <c r="J9" s="19" t="n">
@@ -3262,12 +3262,12 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>North Christina</t>
+          <t>Washington D.C.</t>
         </is>
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>college</t>
+          <t>cold outreach</t>
         </is>
       </c>
       <c r="J10" s="11" t="n">
@@ -3309,12 +3309,12 @@
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>Lisaberg</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
-          <t>college</t>
+          <t>life</t>
         </is>
       </c>
       <c r="J11" s="19" t="n">
@@ -3356,12 +3356,12 @@
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>Johnsonport</t>
+          <t>Washington D.C.</t>
         </is>
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>cold outreach</t>
         </is>
       </c>
       <c r="J12" s="7" t="n"/>
@@ -3401,12 +3401,12 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>West Austinview</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>referral</t>
+          <t>college</t>
         </is>
       </c>
       <c r="J13" s="19" t="n">
@@ -3448,12 +3448,12 @@
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>New Jenniferborough</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>life</t>
+          <t>referral</t>
         </is>
       </c>
       <c r="J14" s="19" t="n">
@@ -3495,12 +3495,12 @@
       </c>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t>Lake Richardfurt</t>
+          <t>Washington D.C.</t>
         </is>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
-          <t>cold outreach</t>
+          <t>life</t>
         </is>
       </c>
       <c r="J15" s="19" t="n">
@@ -3542,12 +3542,12 @@
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>Howardtown</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>life</t>
         </is>
       </c>
       <c r="J16" s="11" t="n">
@@ -3587,12 +3587,12 @@
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>Lake Alexanderland</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>cold outreach</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="J17" s="19" t="n">
@@ -3634,12 +3634,12 @@
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>Elizabethland</t>
+          <t>Washington D.C.</t>
         </is>
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
-          <t>life</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="J18" s="11" t="n">
@@ -3679,12 +3679,12 @@
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>Mcdonaldhaven</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>life</t>
+          <t>other</t>
         </is>
       </c>
       <c r="J19" s="19" t="n">
@@ -3724,12 +3724,12 @@
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>North Michaelview</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>referral</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="J20" s="19" t="n">
@@ -3771,12 +3771,12 @@
       </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>New Danielland</t>
+          <t>Houston</t>
         </is>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>life</t>
         </is>
       </c>
       <c r="J21" s="19" t="n">
@@ -3818,12 +3818,12 @@
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>Jacquelineland</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>life</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="J22" s="11" t="n">
@@ -3865,7 +3865,7 @@
       </c>
       <c r="H23" s="8" t="inlineStr">
         <is>
-          <t>Brendabury</t>
+          <t>Washington D.C.</t>
         </is>
       </c>
       <c r="I23" s="8" t="inlineStr">
@@ -3912,12 +3912,12 @@
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>West Robert</t>
+          <t>Washington D.C.</t>
         </is>
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="J24" s="7" t="n"/>
@@ -3957,7 +3957,7 @@
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>Cooperberg</t>
+          <t>Washington D.C.</t>
         </is>
       </c>
       <c r="I25" s="8" t="inlineStr">
@@ -4004,12 +4004,12 @@
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>Lisahaven</t>
+          <t>Washington D.C.</t>
         </is>
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>cold outreach</t>
+          <t>referral</t>
         </is>
       </c>
       <c r="J26" s="11" t="n">
@@ -4051,12 +4051,12 @@
       </c>
       <c r="H27" s="8" t="inlineStr">
         <is>
-          <t>South Natalie</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
-          <t>cold outreach</t>
+          <t>referral</t>
         </is>
       </c>
       <c r="J27" s="8" t="n"/>
@@ -6416,7 +6416,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="11" t="n">
-        <v>46310</v>
+        <v>45991</v>
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
@@ -6425,12 +6425,12 @@
       </c>
       <c r="E2" s="17" t="inlineStr">
         <is>
-          <t>Enough everybody air nature name.</t>
+          <t>As majority those decide bad answer group.</t>
         </is>
       </c>
       <c r="F2" s="17" t="inlineStr">
         <is>
-          <t>Accept where direction at.</t>
+          <t>Return life raise improve.</t>
         </is>
       </c>
       <c r="G2" s="7" t="n"/>
@@ -6443,7 +6443,7 @@
         <v>4</v>
       </c>
       <c r="C3" s="19" t="n">
-        <v>45676</v>
+        <v>46120</v>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
@@ -6452,12 +6452,12 @@
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>Down store technology enough.</t>
+          <t>Computer fill property down get.</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>After particularly where grow write leave pull trip.</t>
+          <t>Important central cut cause get audience.</t>
         </is>
       </c>
       <c r="G3" s="8" t="n"/>
@@ -6470,21 +6470,21 @@
         <v>7</v>
       </c>
       <c r="C4" s="11" t="n">
-        <v>46377</v>
+        <v>46128</v>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>thank you</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Matter begin third style detail project control.</t>
+          <t>Side foot home show threat recently audience.</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>Mean notice name left.</t>
+          <t>Enter exist close there natural east appear.</t>
         </is>
       </c>
       <c r="G4" s="7" t="n"/>
@@ -6497,16 +6497,16 @@
         <v>7</v>
       </c>
       <c r="C5" s="11" t="n">
-        <v>45794</v>
+        <v>45834</v>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>thank you</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>Like week six maybe seat with.</t>
+          <t>Air nature name yes factor accept where.</t>
         </is>
       </c>
       <c r="F5" s="8" t="n"/>
@@ -6520,21 +6520,21 @@
         <v>8</v>
       </c>
       <c r="C6" s="23" t="n">
-        <v>46348</v>
+        <v>45862</v>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>call</t>
+          <t>thank you</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Similar believe Republican know her involve first clear.</t>
+          <t>Heart down store technology.</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Sound language for child usually trip other.</t>
+          <t>Almost after particularly.</t>
         </is>
       </c>
       <c r="G6" s="7" t="n"/>
@@ -6547,7 +6547,7 @@
         <v>9</v>
       </c>
       <c r="C7" s="19" t="n">
-        <v>45960</v>
+        <v>45729</v>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
@@ -6556,12 +6556,12 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>White suddenly particularly area their stock inside mouth.</t>
+          <t>Spring in interview one fine matter.</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Tend majority blood ago rich piece.</t>
+          <t>Detail project control unit around mean notice name.</t>
         </is>
       </c>
       <c r="G7" s="8" t="n"/>
@@ -6574,21 +6574,21 @@
         <v>10</v>
       </c>
       <c r="C8" s="11" t="n">
-        <v>45689</v>
+        <v>45794</v>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>thank you</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Sea stage somebody keep seek defense offer.</t>
+          <t>Break like week six maybe seat with.</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Structure mean store require position special agree.</t>
+          <t>Similar believe Republican know her involve first clear.</t>
         </is>
       </c>
       <c r="G8" s="7" t="n"/>
@@ -6601,21 +6601,21 @@
         <v>8</v>
       </c>
       <c r="C9" s="19" t="n">
-        <v>46232</v>
+        <v>46102</v>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>Apply action offer ok design fire.</t>
+          <t>Me after middle deep scientist.</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>Three occur painting.</t>
+          <t>Rate up painting save popular other along matter.</t>
         </is>
       </c>
       <c r="G9" s="8" t="n"/>
@@ -6628,16 +6628,16 @@
         <v>9</v>
       </c>
       <c r="C10" s="11" t="n">
-        <v>46204</v>
+        <v>46153</v>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>thank you</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Stock many stage.</t>
+          <t>Inside mouth home himself.</t>
         </is>
       </c>
       <c r="F10" s="7" t="n"/>
@@ -6651,16 +6651,16 @@
         <v>10</v>
       </c>
       <c r="C11" s="19" t="n">
-        <v>46331</v>
+        <v>46235</v>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>call</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Rich treat if different out want.</t>
+          <t>Different three serve read.</t>
         </is>
       </c>
       <c r="F11" s="8" t="n"/>
@@ -6674,21 +6674,21 @@
         <v>11</v>
       </c>
       <c r="C12" s="11" t="n">
-        <v>45885</v>
+        <v>46104</v>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>in person</t>
+          <t>call</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>Late power fill indicate often cell.</t>
+          <t>Somebody keep seek defense.</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Significant race reduce market.</t>
+          <t>Test morning structure.</t>
         </is>
       </c>
       <c r="G12" s="7" t="n"/>
@@ -6701,21 +6701,21 @@
         <v>12</v>
       </c>
       <c r="C13" s="11" t="n">
-        <v>46383</v>
+        <v>45666</v>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>in person</t>
+          <t>thank you</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Beyond pick former same.</t>
+          <t>Word space head case after last apply.</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Rock low professional wrong.</t>
+          <t>Ok design fire.</t>
         </is>
       </c>
       <c r="G13" s="8" t="n"/>
@@ -6728,21 +6728,21 @@
         <v>14</v>
       </c>
       <c r="C14" s="11" t="n">
-        <v>46367</v>
+        <v>45689</v>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>thank you</t>
+          <t>call</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>Practice manager eye foreign history.</t>
+          <t>Three occur painting.</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Ok rate consider leave have office.</t>
+          <t>Candidate center story guess white tend here.</t>
         </is>
       </c>
       <c r="G14" s="7" t="n"/>
@@ -6755,21 +6755,21 @@
         <v>17</v>
       </c>
       <c r="C15" s="11" t="n">
-        <v>45734</v>
+        <v>45964</v>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>in person</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Air into successful lose positive someone there.</t>
+          <t>Out want world arrive suggest.</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Indeed wear hundred Republican finish suffer game.</t>
+          <t>Far agent right policy enter.</t>
         </is>
       </c>
       <c r="G15" s="8" t="n"/>
@@ -6782,21 +6782,21 @@
         <v>13</v>
       </c>
       <c r="C16" s="11" t="n">
-        <v>46091</v>
+        <v>45767</v>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>LinkedIn</t>
+          <t>email</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>Two within director beautiful page.</t>
+          <t>Significant race reduce market.</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>Of wrong run kitchen similar interest front.</t>
+          <t>Pick former same various call fight.</t>
         </is>
       </c>
       <c r="G16" s="7" t="n"/>
@@ -6809,21 +6809,21 @@
         <v>13</v>
       </c>
       <c r="C17" s="19" t="n">
-        <v>46374</v>
+        <v>45879</v>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>call</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>Degree build despite human successful.</t>
+          <t>Professional wrong discuss between environment debate.</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>Pm little walk.</t>
+          <t>Tree game friend treat economic improve child trade.</t>
         </is>
       </c>
       <c r="G17" s="8" t="n"/>
@@ -6836,21 +6836,21 @@
         <v>13</v>
       </c>
       <c r="C18" s="11" t="n">
-        <v>45900</v>
+        <v>45842</v>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>thank you</t>
+          <t>other</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>Probably protect type we student community general.</t>
+          <t>Thought myself usually.</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>Even young suggest happen.</t>
+          <t>Someone there between laugh event allow middle finish.</t>
         </is>
       </c>
       <c r="G18" s="7" t="n"/>
@@ -6863,21 +6863,21 @@
         <v>12</v>
       </c>
       <c r="C19" s="19" t="n">
-        <v>46024</v>
+        <v>46349</v>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>call</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>Scene simple peace them.</t>
+          <t>Suffer game short town two.</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>From system recognize enjoy place possible station senior.</t>
+          <t>Beautiful page newspaper read of wrong run.</t>
         </is>
       </c>
       <c r="G19" s="8" t="n"/>
@@ -6890,21 +6890,21 @@
         <v>21</v>
       </c>
       <c r="C20" s="11" t="n">
-        <v>46170</v>
+        <v>45828</v>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>in person</t>
+          <t>thank you</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>Throw former bar fact mind in.</t>
+          <t>Attorney own movement history degree build.</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>Appear form lot none glass guy city.</t>
+          <t>Low make window whole result analysis.</t>
         </is>
       </c>
       <c r="G20" s="7" t="n"/>
@@ -6917,21 +6917,21 @@
         <v>23</v>
       </c>
       <c r="C21" s="19" t="n">
-        <v>46173</v>
+        <v>46375</v>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>email</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Her as let coach kind.</t>
+          <t>Little walk several probably protect.</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>Doctor mission exactly me just drive.</t>
+          <t>Can instead method even.</t>
         </is>
       </c>
       <c r="G21" s="8" t="n"/>
@@ -6944,21 +6944,21 @@
         <v>23</v>
       </c>
       <c r="C22" s="11" t="n">
-        <v>46213</v>
+        <v>46024</v>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>other</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>Small conference PM white learn animal.</t>
+          <t>Suggest happen size scene simple peace them.</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>Dinner agree shoulder prove water color.</t>
+          <t>From system recognize enjoy place possible station senior.</t>
         </is>
       </c>
       <c r="G22" s="7" t="n"/>
@@ -6971,7 +6971,7 @@
         <v>23</v>
       </c>
       <c r="C23" s="19" t="n">
-        <v>46216</v>
+        <v>46170</v>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
@@ -6980,7 +6980,7 @@
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>Full better hotel nearly answer institution.</t>
+          <t>Throw former bar fact mind in.</t>
         </is>
       </c>
       <c r="F23" s="8" t="n"/>
@@ -6994,16 +6994,16 @@
         <v>25</v>
       </c>
       <c r="C24" s="11" t="n">
-        <v>45928</v>
+        <v>45886</v>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>call</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>Onto near lay.</t>
+          <t>Appear form lot none glass guy city.</t>
         </is>
       </c>
       <c r="F24" s="7" t="n"/>
@@ -7017,16 +7017,16 @@
         <v>24</v>
       </c>
       <c r="C25" s="19" t="n">
-        <v>46247</v>
+        <v>46378</v>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>thank you</t>
+          <t>other</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>Wide two against measure space relate rate.</t>
+          <t>Task rise arrive prevent.</t>
         </is>
       </c>
       <c r="F25" s="8" t="n"/>
@@ -7040,21 +7040,21 @@
         <v>2</v>
       </c>
       <c r="C26" s="11" t="n">
-        <v>45898</v>
+        <v>45961</v>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>call</t>
+          <t>email</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>Most life activity second.</t>
+          <t>Doctor mission exactly me just drive.</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>Help would indeed brother sport at.</t>
+          <t>Visit suggest statement find.</t>
         </is>
       </c>
       <c r="G26" s="7" t="n"/>
@@ -7067,21 +7067,21 @@
         <v>24</v>
       </c>
       <c r="C27" s="19" t="n">
-        <v>45783</v>
+        <v>46255</v>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>call</t>
+          <t>LinkedIn</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>Design over leader indeed.</t>
+          <t>Song dinner agree.</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>Charge spring report take these point east fight.</t>
+          <t>Water color game name you.</t>
         </is>
       </c>
       <c r="G27" s="8" t="n"/>
@@ -7094,16 +7094,16 @@
         <v>24</v>
       </c>
       <c r="C28" s="19" t="n">
-        <v>46031</v>
+        <v>46012</v>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>thank you</t>
+          <t>email</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>Include fly soon voice tree.</t>
+          <t>Every tonight point friend support onto near.</t>
         </is>
       </c>
       <c r="F28" s="8" t="n"/>

</xml_diff>